<commit_message>
Fler sätt att stoppa tvångsbud: lösen, skydd för nyköpt, Motbud, säljarnas marknad
- Lösen: ägaren betalar budgivaren 10 % av MV och behåller fastigheten.
- Fastighet köpt i en marknadsfas kan inte tvångsköpas i samma fas.
- Personkort Motbud (2): stoppar budet och låter ägaren köpa en av budgivarens fastigheter till MV.
- Omvärldskort Säljarnas marknad: tvångsbud till 1,4 × MV vid nästa marknad.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_omvärldskort.xlsx
+++ b/kortdata/F_omvärldskort.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1742,6 +1742,44 @@
         </is>
       </c>
       <c r="H36" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>OM-36</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>saljares_marknad</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>1,4</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>alla</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Kapitalet flödar — säljarnas marknad</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Alla vill köpa, ingen vill sälja. Alla tvångsbud vid nästa marknad kostar 1,4 × MV i stället för 1,2 × MV.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1792,7 +1830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2337,6 +2375,21 @@
         </is>
       </c>
       <c r="C36" t="inlineStr">
+        <is>
+          <t>ej bestämt</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Kapitalet flödar — säljarnas marknad</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
         <is>
           <t>ej bestämt</t>
         </is>
@@ -2610,7 +2663,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>35 (kortspecen: 35)</t>
+          <t>36 (kortspecen: 36)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Omvärldskorten flyttar yielden direkt – yieldbanan ändras aldrig
Beslut (Niklas): kort ska inte byta effekt på andra kort. De 23 yieldkorten bland
omvärldskorten ('lägg kortet på nästa plats', 'byt ut nästa/alla yieldkort') flyttar nu
yielden direkt ±0,5 på ett eller båda spåren (ny effekt yield_nu); yieldbanan som lades vid
start ligger kvar som den är. De sex 'byt ut'-korten fick en fast riktning efter rubriken.
Regelboken 9.10. 400 partier: förvaltningsstrategierna 23–27 %. Tryckfilen byggd om.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_omvärldskort.xlsx
+++ b/kortdata/F_omvärldskort.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Styrräntan höjs oväntat mer än marknaden räknat med. Gäller nu: lägg kortet på nästa plats på bostadsspåret (+0,5 procentenheter).</t>
+          <t>Styrräntan höjs oväntat mer än marknaden räknat med. Direkt: yielden på bostadsspåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -536,7 +536,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Institutionellt kapital söker sig till andra tillgångsslag. Gäller nu: lägg kortet på nästa plats på bostadsspåret (+0,5 procentenheter).</t>
+          <t>Institutionellt kapital söker sig till andra tillgångsslag. Direkt: yielden på bostadsspåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -574,7 +574,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nya krav på hushållens amortering kyler ner bostadsmarknaden. Gäller nu: lägg kortet på nästa plats på bostadsspåret (+0,5 procentenheter).</t>
+          <t>Nya krav på hushållens amortering kyler ner bostadsmarknaden. Direkt: yielden på bostadsspåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -612,7 +612,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sänkt styrränta lättar trycket på fastighetsägarna. Gäller nu: lägg kortet på nästa plats på bostadsspåret (-0,5 procentenheter).</t>
+          <t>Sänkt styrränta lättar trycket på fastighetsägarna. Direkt: yielden på bostadsspåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -650,7 +650,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Nyproduktionen halkar efter befolkningstillväxten. Gäller nu: lägg kortet på nästa plats på bostadsspåret (-0,5 procentenheter).</t>
+          <t>Nyproduktionen halkar efter befolkningstillväxten. Direkt: yielden på bostadsspåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -688,7 +688,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Pensionsfonder ökar sina placeringar i svenska bostäder. Gäller nu: lägg kortet på nästa plats på bostadsspåret (-0,5 procentenheter).</t>
+          <t>Pensionsfonder ökar sina placeringar i svenska bostäder. Direkt: yielden på bostadsspåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Fler företag säger upp kontorsyta de inte längre behöver. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (+0,5 procentenheter).</t>
+          <t>Fler företag säger upp kontorsyta de inte längre behöver. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -764,7 +764,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Butiker och restauranger drar ner på nyetableringar. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (+0,5 procentenheter).</t>
+          <t>Butiker och restauranger drar ner på nyetableringar. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -802,7 +802,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Kontorsytor i centrala lägen står tomma allt längre. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (+0,5 procentenheter).</t>
+          <t>Kontorsytor i centrala lägen står tomma allt längre. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -840,7 +840,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Nyetableringar fyller lediga kontorsytor snabbare än väntat. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (-0,5 procentenheter).</t>
+          <t>Nyetableringar fyller lediga kontorsytor snabbare än väntat. Direkt: yielden på det kommersiella spåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -878,7 +878,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Efterfrågan på lager och logistikytor ökar kraftigt. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (-0,5 procentenheter).</t>
+          <t>Efterfrågan på lager och logistikytor ökar kraftigt. Direkt: yielden på det kommersiella spåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -916,7 +916,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Utländska investerare ökar sina bud på svenska kontorsfastigheter. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (-0,5 procentenheter).</t>
+          <t>Utländska investerare ökar sina bud på svenska kontorsfastigheter. Direkt: yielden på det kommersiella spåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -954,7 +954,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Byggtakten har inte hängt med på flera år och trycket på hyresmarknaden är akut. Gäller nu: lägg kortet på nästa plats på bostadsspåret (-0,5 procentenheter).</t>
+          <t>Byggtakten har inte hängt med på flera år och trycket på hyresmarknaden är akut. Direkt: yielden på bostadsspåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -992,7 +992,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Kreditmarknaden stramas åt och investerare drar sig från kommersiella fastigheter. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (+0,5 procentenheter).</t>
+          <t>Kreditmarknaden stramas åt och investerare drar sig från kommersiella fastigheter. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>En snabb och kraftig räntehöjning skakar om hela bostadssektorn. Gäller nu: lägg kortet på nästa plats på bostadsspåret (+0,5 procentenheter).</t>
+          <t>En snabb och kraftig räntehöjning skakar om hela bostadssektorn. Direkt: yielden på bostadsspåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1306,10 +1306,14 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>yield_byt</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
+          <t>yield_nu</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>+0,5</t>
+        </is>
+      </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>bostäder</t>
@@ -1322,7 +1326,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Bedömarna är oense om vart bostadspriserna är på väg. Byt ut: ersätt nästa yieldkort på bostadsspåret med det översta kortet ur yieldleken.</t>
+          <t>Bedömarna är oense och köparna avvaktar. Direkt: yielden på bostadsspåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
@@ -1340,10 +1344,14 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>yield_byt</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
+          <t>yield_nu</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>+0,5</t>
+        </is>
+      </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
           <t>kommersiellt</t>
@@ -1356,7 +1364,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Värderingsinstituten ser över sina antaganden för kontor och handel. Byt ut: ersätt nästa yieldkort på det kommersiella spåret med det översta kortet ur yieldleken.</t>
+          <t>Värderingsinstituten skriver ned sina antaganden för kontor och handel. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
@@ -1374,10 +1382,14 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>yield_byt</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
+          <t>yield_nu</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>-0,5</t>
+        </is>
+      </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
           <t>båda</t>
@@ -1390,7 +1402,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Storbankens analytiker skriver om hela sin fastighetsprognos. Byt ut: ersätt nästa yieldkort på både bostadsspåret och det kommersiella spåret med det översta kortet ur yieldleken.</t>
+          <t>Storbankens analytiker skriver upp hela sin fastighetsprognos. Direkt: yielden på båda spåren sjunker 0,5 procentenheter (flytta markörerna). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
@@ -1408,10 +1420,14 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>yield_byt</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
+          <t>yield_nu</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>+0,5</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
           <t>båda</t>
@@ -1424,7 +1440,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Ett regeringsskifte gör framtiden svårläst för investerarna. Byt ut: ersätt nästa yieldkort på både bostadsspåret och det kommersiella spåret med det översta kortet ur yieldleken.</t>
+          <t>Ett regeringsskifte gör framtiden svårläst och investerarna kräver mer. Direkt: yielden på båda spåren stiger 0,5 procentenheter (flytta markörerna). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
@@ -1442,10 +1458,14 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>yield_byt_alla</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
+          <t>yield_nu</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>-0,5</t>
+        </is>
+      </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>bostäder</t>
@@ -1458,7 +1478,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Regeringen lägger om hela bostadspolitiken. Byt ut alla kvarvarande yieldkort på bostadsspåret mot nya ur yieldleken.</t>
+          <t>Regeringen lägger om bostadspolitiken till förmån för hyresrätter. Direkt: yielden på bostadsspåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
@@ -1476,10 +1496,14 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>yield_byt_alla</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr"/>
+          <t>yield_nu</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>+0,5</t>
+        </is>
+      </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
           <t>kommersiellt</t>
@@ -1492,7 +1516,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Arbetsliv och handel förändras i grunden. Byt ut alla kvarvarande yieldkort på det kommersiella spåret mot nya ur yieldleken.</t>
+          <t>Arbetsliv och handel förändras i grunden, och kontorsbehovet krymper. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H29" s="2" t="n">
@@ -1718,7 +1742,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1738,7 +1762,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Säljarna är nervösa och priserna faller. Gäller nu: lägg kortet på nästa plats på båda spåren (+0,5 procentenheter).</t>
+          <t>Säljarna är nervösa och priserna faller. Direkt: yielden på båda spåren stiger 0,5 procentenheter (flytta markörerna). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
@@ -1756,7 +1780,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>yield_ersatt</t>
+          <t>yield_nu</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1776,7 +1800,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Alla vill köpa, ingen vill sälja, och priserna stiger. Gäller nu: lägg kortet på nästa plats på båda spåren (−0,5 procentenheter).</t>
+          <t>Alla vill köpa, ingen vill sälja, och priserna stiger. Direkt: yielden på båda spåren sjunker 0,5 procentenheter (flytta markörerna). Yieldbanan ändras inte.</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">

</xml_diff>

<commit_message>
Återställ: omvärldskortens yieldkort läggs på yieldbanan som förut
Beslut (Niklas): yielden ska fungera som förut – 'lägg kortet på nästa plats' och 'byt ut'
gäller igen (reverts fc07253). OM-35/36 förblir yieldkort på båda spåren.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_omvärldskort.xlsx
+++ b/kortdata/F_omvärldskort.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Styrräntan höjs oväntat mer än marknaden räknat med. Direkt: yielden på bostadsspåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Styrräntan höjs oväntat mer än marknaden räknat med. Gäller nu: lägg kortet på nästa plats på bostadsspåret (+0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -536,7 +536,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Institutionellt kapital söker sig till andra tillgångsslag. Direkt: yielden på bostadsspåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Institutionellt kapital söker sig till andra tillgångsslag. Gäller nu: lägg kortet på nästa plats på bostadsspåret (+0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -574,7 +574,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nya krav på hushållens amortering kyler ner bostadsmarknaden. Direkt: yielden på bostadsspåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Nya krav på hushållens amortering kyler ner bostadsmarknaden. Gäller nu: lägg kortet på nästa plats på bostadsspåret (+0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -612,7 +612,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sänkt styrränta lättar trycket på fastighetsägarna. Direkt: yielden på bostadsspåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Sänkt styrränta lättar trycket på fastighetsägarna. Gäller nu: lägg kortet på nästa plats på bostadsspåret (-0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -650,7 +650,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Nyproduktionen halkar efter befolkningstillväxten. Direkt: yielden på bostadsspåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Nyproduktionen halkar efter befolkningstillväxten. Gäller nu: lägg kortet på nästa plats på bostadsspåret (-0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -688,7 +688,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Pensionsfonder ökar sina placeringar i svenska bostäder. Direkt: yielden på bostadsspåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Pensionsfonder ökar sina placeringar i svenska bostäder. Gäller nu: lägg kortet på nästa plats på bostadsspåret (-0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Fler företag säger upp kontorsyta de inte längre behöver. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Fler företag säger upp kontorsyta de inte längre behöver. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (+0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -764,7 +764,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Butiker och restauranger drar ner på nyetableringar. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Butiker och restauranger drar ner på nyetableringar. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (+0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -802,7 +802,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Kontorsytor i centrala lägen står tomma allt längre. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Kontorsytor i centrala lägen står tomma allt längre. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (+0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -840,7 +840,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Nyetableringar fyller lediga kontorsytor snabbare än väntat. Direkt: yielden på det kommersiella spåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Nyetableringar fyller lediga kontorsytor snabbare än väntat. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (-0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -878,7 +878,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Efterfrågan på lager och logistikytor ökar kraftigt. Direkt: yielden på det kommersiella spåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Efterfrågan på lager och logistikytor ökar kraftigt. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (-0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -916,7 +916,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Utländska investerare ökar sina bud på svenska kontorsfastigheter. Direkt: yielden på det kommersiella spåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Utländska investerare ökar sina bud på svenska kontorsfastigheter. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (-0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -954,7 +954,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Byggtakten har inte hängt med på flera år och trycket på hyresmarknaden är akut. Direkt: yielden på bostadsspåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Byggtakten har inte hängt med på flera år och trycket på hyresmarknaden är akut. Gäller nu: lägg kortet på nästa plats på bostadsspåret (-0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -992,7 +992,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Kreditmarknaden stramas åt och investerare drar sig från kommersiella fastigheter. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Kreditmarknaden stramas åt och investerare drar sig från kommersiella fastigheter. Gäller nu: lägg kortet på nästa plats på det kommersiella spåret (+0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>En snabb och kraftig räntehöjning skakar om hela bostadssektorn. Direkt: yielden på bostadsspåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>En snabb och kraftig räntehöjning skakar om hela bostadssektorn. Gäller nu: lägg kortet på nästa plats på bostadsspåret (+0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1306,14 +1306,10 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>+0,5</t>
-        </is>
-      </c>
+          <t>yield_byt</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>bostäder</t>
@@ -1326,7 +1322,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Bedömarna är oense och köparna avvaktar. Direkt: yielden på bostadsspåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Bedömarna är oense om vart bostadspriserna är på väg. Byt ut: ersätt nästa yieldkort på bostadsspåret med det översta kortet ur yieldleken.</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
@@ -1344,14 +1340,10 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>+0,5</t>
-        </is>
-      </c>
+          <t>yield_byt</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr">
         <is>
           <t>kommersiellt</t>
@@ -1364,7 +1356,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Värderingsinstituten skriver ned sina antaganden för kontor och handel. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Värderingsinstituten ser över sina antaganden för kontor och handel. Byt ut: ersätt nästa yieldkort på det kommersiella spåret med det översta kortet ur yieldleken.</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
@@ -1382,14 +1374,10 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>-0,5</t>
-        </is>
-      </c>
+          <t>yield_byt</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
           <t>båda</t>
@@ -1402,7 +1390,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Storbankens analytiker skriver upp hela sin fastighetsprognos. Direkt: yielden på båda spåren sjunker 0,5 procentenheter (flytta markörerna). Yieldbanan ändras inte.</t>
+          <t>Storbankens analytiker skriver om hela sin fastighetsprognos. Byt ut: ersätt nästa yieldkort på både bostadsspåret och det kommersiella spåret med det översta kortet ur yieldleken.</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
@@ -1420,14 +1408,10 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>+0,5</t>
-        </is>
-      </c>
+          <t>yield_byt</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr">
         <is>
           <t>båda</t>
@@ -1440,7 +1424,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Ett regeringsskifte gör framtiden svårläst och investerarna kräver mer. Direkt: yielden på båda spåren stiger 0,5 procentenheter (flytta markörerna). Yieldbanan ändras inte.</t>
+          <t>Ett regeringsskifte gör framtiden svårläst för investerarna. Byt ut: ersätt nästa yieldkort på både bostadsspåret och det kommersiella spåret med det översta kortet ur yieldleken.</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
@@ -1458,14 +1442,10 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>-0,5</t>
-        </is>
-      </c>
+          <t>yield_byt_alla</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>bostäder</t>
@@ -1478,7 +1458,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Regeringen lägger om bostadspolitiken till förmån för hyresrätter. Direkt: yielden på bostadsspåret sjunker 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Regeringen lägger om hela bostadspolitiken. Byt ut alla kvarvarande yieldkort på bostadsspåret mot nya ur yieldleken.</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
@@ -1496,14 +1476,10 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>+0,5</t>
-        </is>
-      </c>
+          <t>yield_byt_alla</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr">
         <is>
           <t>kommersiellt</t>
@@ -1516,7 +1492,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Arbetsliv och handel förändras i grunden, och kontorsbehovet krymper. Direkt: yielden på det kommersiella spåret stiger 0,5 procentenheter (flytta markören). Yieldbanan ändras inte.</t>
+          <t>Arbetsliv och handel förändras i grunden. Byt ut alla kvarvarande yieldkort på det kommersiella spåret mot nya ur yieldleken.</t>
         </is>
       </c>
       <c r="H29" s="2" t="n">
@@ -1742,7 +1718,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1762,7 +1738,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Säljarna är nervösa och priserna faller. Direkt: yielden på båda spåren stiger 0,5 procentenheter (flytta markörerna). Yieldbanan ändras inte.</t>
+          <t>Säljarna är nervösa och priserna faller. Gäller nu: lägg kortet på nästa plats på båda spåren (+0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
@@ -1780,7 +1756,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>yield_nu</t>
+          <t>yield_ersatt</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1800,7 +1776,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Alla vill köpa, ingen vill sälja, och priserna stiger. Direkt: yielden på båda spåren sjunker 0,5 procentenheter (flytta markörerna). Yieldbanan ändras inte.</t>
+          <t>Alla vill köpa, ingen vill sälja, och priserna stiger. Gäller nu: lägg kortet på nästa plats på båda spåren (−0,5 procentenheter).</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">

</xml_diff>